<commit_message>
fix. problem with old ref. and bad namespace after orchestrator and studio update
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA\Theresia\RPA-ArvoderadeUppdrag\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA\Oskar\RPA-ArvoderadeUppdrag\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD3E87C-A793-4532-91A2-4402CDFAAE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" activeTab="2"/>
+    <workbookView xWindow="690" yWindow="2730" windowWidth="38700" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="67">
   <si>
     <t>Name</t>
   </si>
@@ -222,12 +223,15 @@
   </si>
   <si>
     <t>OkNrOfMonthBack</t>
+  </si>
+  <si>
+    <t>FolderPathOrch</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5">
     <font>
       <sz val="11"/>
@@ -606,7 +610,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z997"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -698,7 +702,9 @@
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" s="4"/>
+      <c r="A7" s="4" t="s">
+        <v>66</v>
+      </c>
       <c r="B7" s="4"/>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1699,7 +1705,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z989"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -2864,7 +2870,7 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
@@ -2872,7 +2878,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z995"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>

</xml_diff>